<commit_message>
Repo Updates post revision
</commit_message>
<xml_diff>
--- a/R_Codes/DataSummary/All_Prokaryotes/Sample_Layer/All_Prokaryotes_Summary_Domain_by_Sample_Layer.xlsx
+++ b/R_Codes/DataSummary/All_Prokaryotes/Sample_Layer/All_Prokaryotes_Summary_Domain_by_Sample_Layer.xlsx
@@ -484,10 +484,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>90.2962078272753</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.445187403589909</v>
+        <v>90.2972806732504</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.445414314580794</v>
       </c>
     </row>
     <row r="3">
@@ -498,10 +498,10 @@
         <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>9.70379217272427</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.0930725858884609</v>
+        <v>9.70271932675006</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.0930752015502293</v>
       </c>
     </row>
   </sheetData>
@@ -537,10 +537,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>75.8975809766081</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.294769321127961</v>
+        <v>75.8954334159013</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.294988349534254</v>
       </c>
     </row>
     <row r="3">
@@ -551,10 +551,10 @@
         <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>24.1024190233925</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.213589472786736</v>
+        <v>24.1045665840983</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.213601767670852</v>
       </c>
     </row>
   </sheetData>
@@ -643,10 +643,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>64.6884792988097</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.189215394833972</v>
+        <v>64.6884262516967</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.189350278554429</v>
       </c>
     </row>
     <row r="3">
@@ -657,10 +657,10 @@
         <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>35.3115207011892</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.410284361255583</v>
+        <v>35.3115737483024</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.410278563326449</v>
       </c>
     </row>
   </sheetData>
@@ -696,10 +696,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>90.410842719501</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.436242734937012</v>
+        <v>90.4115024979413</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.436555315909587</v>
       </c>
     </row>
     <row r="3">
@@ -710,10 +710,10 @@
         <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>9.58915728049938</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.185917934650432</v>
+        <v>9.58849750205889</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.185905819925326</v>
       </c>
     </row>
   </sheetData>
@@ -749,10 +749,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>85.0834701892304</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.426031443115377</v>
+        <v>85.0790101864731</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.426431789232129</v>
       </c>
     </row>
     <row r="3">
@@ -763,10 +763,10 @@
         <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>14.9165298107707</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.5737011727746</v>
+        <v>14.9209898135273</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.574062566507061</v>
       </c>
     </row>
   </sheetData>
@@ -802,10 +802,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>64.686091291812</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.209901988344044</v>
+        <v>64.6734140482954</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.210173734038262</v>
       </c>
     </row>
     <row r="3">
@@ -816,10 +816,10 @@
         <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>35.313908708188</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.809010296217597</v>
+        <v>35.326585951704</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.809263423807461</v>
       </c>
     </row>
   </sheetData>
@@ -908,10 +908,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>70.3461830234325</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.592986929187446</v>
+        <v>70.3445744478286</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.593527876192317</v>
       </c>
     </row>
     <row r="3">
@@ -922,10 +922,10 @@
         <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>29.6538169765681</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.21476735840129</v>
+        <v>29.6554255521717</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.214823658381749</v>
       </c>
     </row>
   </sheetData>
@@ -961,10 +961,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>98.1424007653047</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2.84628817050189</v>
+        <v>98.1966990907347</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2.81993688368827</v>
       </c>
     </row>
     <row r="3">
@@ -975,10 +975,10 @@
         <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>1.85759923469527</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.427715942019033</v>
+        <v>1.80330090926535</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.415213633124304</v>
       </c>
     </row>
   </sheetData>
@@ -1014,10 +1014,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>54.1024185606343</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1.61454419402737</v>
+        <v>52.803510496473</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.66160302386933</v>
       </c>
     </row>
     <row r="3">
@@ -1028,10 +1028,10 @@
         <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>45.8975814393654</v>
-      </c>
-      <c r="D3" t="n">
-        <v>3.25413247818942</v>
+        <v>47.1964895035269</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3.34685285317104</v>
       </c>
     </row>
   </sheetData>
@@ -1067,10 +1067,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>84.6582468642362</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.324873722482319</v>
+        <v>84.6608460896988</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.325207124870217</v>
       </c>
     </row>
     <row r="3">
@@ -1081,10 +1081,10 @@
         <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>15.3417531357648</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.137643981046964</v>
+        <v>15.3391539103035</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.137627687773578</v>
       </c>
     </row>
   </sheetData>

</xml_diff>